<commit_message>
Graphify Update y catalogov2
</commit_message>
<xml_diff>
--- a/pm4-app/insumos/CATALOGOS v2.xlsx
+++ b/pm4-app/insumos/CATALOGOS v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\DockerProys\CLAUDEPM4Copia\pm4-app\insumos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B97F81B1-55BD-4830-8BAA-AB93BBD42527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6392A821-5A41-467B-91E4-A241127DDCEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32850" yWindow="3150" windowWidth="21600" windowHeight="11295" xr2:uid="{AF2F6A33-F3FA-4B8F-93FF-FFB32AF9C232}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{AF2F6A33-F3FA-4B8F-93FF-FFB32AF9C232}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -577,7 +577,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -604,8 +604,15 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -615,6 +622,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDAE9F8"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -631,7 +644,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -645,6 +658,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1301,7 +1316,7 @@
       <c r="C33" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E33" s="1"/>
@@ -1661,10 +1676,10 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
-      <c r="B67" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C67" s="2" t="s">
+      <c r="B67" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>57</v>
       </c>
       <c r="D67" s="1"/>

</xml_diff>